<commit_message>
Atualiza fluxo: XML sempre + fechamento não bloqueante + logs prestados
</commit_message>
<xml_diff>
--- a/empresas.xlsx
+++ b/empresas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows 11\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Windows 11\Desktop\NFS XML\automacao-nfse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9DA73C3-C95D-4118-A8E5-88257C482F24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41CB5EC5-38C5-41CE-97D6-0BCDB6207E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{91D0C60C-AB4A-44B4-A589-DD4A23F71BC5}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="854" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="331">
   <si>
     <t>EMPRESAS SIMPLES NACIONAL</t>
   </si>
@@ -113,19 +113,10 @@
     <t>24.125.988.0001-83</t>
   </si>
   <si>
-    <t>14.128.421.0003-79</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
     <t>14.128.421.0001-07</t>
-  </si>
-  <si>
-    <t>A. P. G. TOP 20 - [(MG) MATRIZ]</t>
-  </si>
-  <si>
-    <t>58.150.107.0001-04</t>
   </si>
   <si>
     <t>AKIKO OKA   (NOTA MANUAL)</t>
@@ -1095,9 +1086,6 @@
   </si>
   <si>
     <t>NÃO</t>
-  </si>
-  <si>
-    <t>A. P. G. COM. - FILIAL - MG - UBERLANDIA    MANDAR NO WHATS</t>
   </si>
   <si>
     <t>A. P. G. COM. COL. LTDA (manda  arquivo) MANDAR NO WHATS</t>
@@ -2012,7 +2000,7 @@
         <v>11</v>
       </c>
       <c r="L2" s="80" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="M2" s="80"/>
       <c r="N2" s="81"/>
@@ -2060,15 +2048,15 @@
         <v>1847</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G5" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H5" s="31"/>
       <c r="I5" s="31"/>
       <c r="J5" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K5" s="31"/>
     </row>
@@ -2089,15 +2077,15 @@
         <v>1847</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H6" s="31"/>
       <c r="I6" s="31"/>
       <c r="J6" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K6" s="31"/>
     </row>
@@ -2118,15 +2106,15 @@
         <v>1847</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H7" s="31"/>
       <c r="I7" s="31"/>
       <c r="J7" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K7" s="31"/>
     </row>
@@ -2147,15 +2135,15 @@
         <v>1847</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H8" s="31"/>
       <c r="I8" s="31"/>
       <c r="J8" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K8" s="31"/>
     </row>
@@ -2163,15 +2151,9 @@
       <c r="A9" s="41">
         <v>913</v>
       </c>
-      <c r="B9" s="42" t="s">
-        <v>309</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="44" t="s">
-        <v>17</v>
-      </c>
+      <c r="B9" s="42"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="45"/>
       <c r="F9" s="46"/>
       <c r="G9" s="46"/>
@@ -2185,10 +2167,10 @@
         <v>413</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="33" t="s">
         <v>17</v>
@@ -2197,15 +2179,15 @@
         <v>1847</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H10" s="31"/>
       <c r="I10" s="31"/>
       <c r="J10" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K10" s="31"/>
     </row>
@@ -2213,15 +2195,9 @@
       <c r="A11" s="41">
         <v>1008</v>
       </c>
-      <c r="B11" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="43" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="44" t="s">
-        <v>17</v>
-      </c>
+      <c r="B11" s="42"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="44"/>
       <c r="E11" s="45"/>
       <c r="F11" s="46"/>
       <c r="G11" s="46"/>
@@ -2235,10 +2211,10 @@
         <v>947</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C12" s="50" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D12" s="51" t="s">
         <v>20</v>
@@ -2247,15 +2223,15 @@
         <v>184718</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H12" s="31"/>
       <c r="I12" s="31"/>
       <c r="J12" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K12" s="31"/>
     </row>
@@ -2264,10 +2240,10 @@
         <v>901</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C13" s="29" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>14</v>
@@ -2276,15 +2252,15 @@
         <v>184718</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H13" s="31"/>
       <c r="I13" s="31"/>
       <c r="J13" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K13" s="31"/>
     </row>
@@ -2293,19 +2269,19 @@
         <v>926</v>
       </c>
       <c r="B14" s="54" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="C14" s="55" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" s="53" t="s">
         <v>17</v>
       </c>
       <c r="E14" s="56" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F14" s="46" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G14" s="46"/>
       <c r="H14" s="46"/>
@@ -2318,19 +2294,19 @@
         <v>1042</v>
       </c>
       <c r="B15" s="54" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C15" s="55" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D15" s="53" t="s">
         <v>14</v>
       </c>
       <c r="E15" s="57" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F15" s="46" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="G15" s="46"/>
       <c r="H15" s="46"/>
@@ -2343,10 +2319,10 @@
         <v>366</v>
       </c>
       <c r="B16" s="28" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>14</v>
@@ -2355,15 +2331,15 @@
         <v>1847</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H16" s="31"/>
       <c r="I16" s="31"/>
       <c r="J16" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K16" s="31"/>
     </row>
@@ -2372,10 +2348,10 @@
         <v>940</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C17" s="29" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D17" s="33" t="s">
         <v>17</v>
@@ -2384,15 +2360,15 @@
         <v>1847</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H17" s="31"/>
       <c r="I17" s="31"/>
       <c r="J17" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K17" s="31"/>
     </row>
@@ -2401,10 +2377,10 @@
         <v>823</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D18" s="61" t="s">
         <v>14</v>
@@ -2413,15 +2389,15 @@
         <v>1847</v>
       </c>
       <c r="F18" s="63" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G18" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H18" s="63"/>
       <c r="I18" s="63"/>
       <c r="J18" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K18" s="63"/>
     </row>
@@ -2430,10 +2406,10 @@
         <v>1002</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D19" s="20" t="s">
         <v>14</v>
@@ -2442,15 +2418,15 @@
         <v>1847</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H19" s="31"/>
       <c r="I19" s="31"/>
       <c r="J19" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K19" s="31"/>
     </row>
@@ -2459,27 +2435,27 @@
         <v>754</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D20" s="33" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E20" s="34">
         <v>184718</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H20" s="31"/>
       <c r="I20" s="31"/>
       <c r="J20" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K20" s="31"/>
     </row>
@@ -2488,10 +2464,10 @@
         <v>395</v>
       </c>
       <c r="B21" s="28" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C21" s="29" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D21" s="20" t="s">
         <v>14</v>
@@ -2500,15 +2476,15 @@
         <v>1847</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H21" s="31"/>
       <c r="I21" s="31"/>
       <c r="J21" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K21" s="31"/>
     </row>
@@ -2517,10 +2493,10 @@
         <v>90</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D22" s="20" t="s">
         <v>17</v>
@@ -2529,15 +2505,15 @@
         <v>1847</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H22" s="31"/>
       <c r="I22" s="31"/>
       <c r="J22" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K22" s="31"/>
     </row>
@@ -2546,10 +2522,10 @@
         <v>541</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D23" s="20" t="s">
         <v>14</v>
@@ -2558,15 +2534,15 @@
         <v>1847</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H23" s="31"/>
       <c r="I23" s="31"/>
       <c r="J23" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K23" s="31"/>
     </row>
@@ -2575,10 +2551,10 @@
         <v>726</v>
       </c>
       <c r="B24" s="49" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>14</v>
@@ -2587,15 +2563,15 @@
         <v>1847</v>
       </c>
       <c r="F24" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H24" s="31"/>
       <c r="I24" s="31"/>
       <c r="J24" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K24" s="31"/>
     </row>
@@ -2604,10 +2580,10 @@
         <v>900</v>
       </c>
       <c r="B25" s="49" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D25" s="20" t="s">
         <v>17</v>
@@ -2616,15 +2592,15 @@
         <v>184718</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H25" s="31"/>
       <c r="I25" s="31"/>
       <c r="J25" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K25" s="31"/>
     </row>
@@ -2633,10 +2609,10 @@
         <v>887</v>
       </c>
       <c r="B26" s="65" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C26" s="66" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D26" s="58" t="s">
         <v>17</v>
@@ -2645,15 +2621,15 @@
         <v>184718</v>
       </c>
       <c r="F26" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G26" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H26" s="31"/>
       <c r="I26" s="31"/>
       <c r="J26" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K26" s="31"/>
     </row>
@@ -2662,10 +2638,10 @@
         <v>959</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C27" s="68" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D27" s="20" t="s">
         <v>17</v>
@@ -2674,15 +2650,15 @@
         <v>1847</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G27" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H27" s="31"/>
       <c r="I27" s="31"/>
       <c r="J27" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K27" s="31"/>
     </row>
@@ -2691,10 +2667,10 @@
         <v>1045</v>
       </c>
       <c r="B28" s="49" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C28" s="68" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D28" s="20" t="s">
         <v>20</v>
@@ -2703,15 +2679,15 @@
         <v>1847</v>
       </c>
       <c r="F28" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G28" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H28" s="31"/>
       <c r="I28" s="31"/>
       <c r="J28" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K28" s="31"/>
     </row>
@@ -2720,10 +2696,10 @@
         <v>388</v>
       </c>
       <c r="B29" s="28" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D29" s="20" t="s">
         <v>14</v>
@@ -2732,15 +2708,15 @@
         <v>1847</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H29" s="31"/>
       <c r="I29" s="31"/>
       <c r="J29" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K29" s="31"/>
     </row>
@@ -2749,10 +2725,10 @@
         <v>729</v>
       </c>
       <c r="B30" s="28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D30" s="20" t="s">
         <v>20</v>
@@ -2761,15 +2737,15 @@
         <v>1847</v>
       </c>
       <c r="F30" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G30" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H30" s="31"/>
       <c r="I30" s="31"/>
       <c r="J30" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K30" s="31"/>
     </row>
@@ -2778,10 +2754,10 @@
         <v>960</v>
       </c>
       <c r="B31" s="51" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C31" s="50" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D31" s="20" t="s">
         <v>14</v>
@@ -2790,19 +2766,19 @@
         <v>184718</v>
       </c>
       <c r="F31" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H31" s="31"/>
       <c r="I31" s="31"/>
       <c r="J31" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K31" s="31"/>
       <c r="L31" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="32" spans="1:12" s="70" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2810,10 +2786,10 @@
         <v>839</v>
       </c>
       <c r="B32" s="49" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D32" s="20" t="s">
         <v>14</v>
@@ -2822,15 +2798,15 @@
         <v>1847</v>
       </c>
       <c r="F32" s="69" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G32" s="69" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H32" s="69"/>
       <c r="I32" s="69"/>
       <c r="J32" s="69" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K32" s="69"/>
       <c r="L32" s="71"/>
@@ -2840,10 +2816,10 @@
         <v>733</v>
       </c>
       <c r="B33" s="28" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>14</v>
@@ -2852,15 +2828,15 @@
         <v>184718</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G33" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H33" s="31"/>
       <c r="I33" s="31"/>
       <c r="J33" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K33" s="31"/>
     </row>
@@ -2884,10 +2860,10 @@
         <v>85</v>
       </c>
       <c r="B35" s="49" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C35" s="33" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D35" s="20" t="s">
         <v>14</v>
@@ -2896,15 +2872,15 @@
         <v>1847</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G35" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H35" s="31"/>
       <c r="I35" s="31"/>
       <c r="J35" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K35" s="31"/>
     </row>
@@ -2913,10 +2889,10 @@
         <v>47</v>
       </c>
       <c r="B36" s="49" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C36" s="33" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D36" s="20" t="s">
         <v>14</v>
@@ -2925,15 +2901,15 @@
         <v>2252</v>
       </c>
       <c r="F36" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G36" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H36" s="31"/>
       <c r="I36" s="31"/>
       <c r="J36" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K36" s="31"/>
     </row>
@@ -2942,10 +2918,10 @@
         <v>50</v>
       </c>
       <c r="B37" s="28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D37" s="20" t="s">
         <v>14</v>
@@ -2954,15 +2930,15 @@
         <v>1847</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G37" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H37" s="31"/>
       <c r="I37" s="31"/>
       <c r="J37" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K37" s="31"/>
     </row>
@@ -2971,10 +2947,10 @@
         <v>434</v>
       </c>
       <c r="B38" s="49" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C38" s="33" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D38" s="20" t="s">
         <v>14</v>
@@ -2983,15 +2959,15 @@
         <v>1847</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G38" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H38" s="31"/>
       <c r="I38" s="31"/>
       <c r="J38" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K38" s="31"/>
     </row>
@@ -3000,10 +2976,10 @@
         <v>244</v>
       </c>
       <c r="B39" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D39" s="20" t="s">
         <v>20</v>
@@ -3012,19 +2988,19 @@
         <v>1847</v>
       </c>
       <c r="F39" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G39" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H39" s="31"/>
       <c r="I39" s="31"/>
       <c r="J39" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K39" s="31"/>
       <c r="L39" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="40" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3032,10 +3008,10 @@
         <v>167</v>
       </c>
       <c r="B40" s="28" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D40" s="20" t="s">
         <v>14</v>
@@ -3044,15 +3020,15 @@
         <v>1847</v>
       </c>
       <c r="F40" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G40" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H40" s="31"/>
       <c r="I40" s="31"/>
       <c r="J40" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K40" s="31"/>
     </row>
@@ -3061,10 +3037,10 @@
         <v>824</v>
       </c>
       <c r="B41" s="49" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D41" s="20" t="s">
         <v>14</v>
@@ -3073,19 +3049,19 @@
         <v>1847</v>
       </c>
       <c r="F41" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H41" s="31"/>
       <c r="I41" s="31"/>
       <c r="J41" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K41" s="31"/>
       <c r="L41" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="42" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3093,10 +3069,10 @@
         <v>812</v>
       </c>
       <c r="B42" s="49" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D42" s="20" t="s">
         <v>14</v>
@@ -3105,19 +3081,19 @@
         <v>1847</v>
       </c>
       <c r="F42" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G42" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H42" s="31"/>
       <c r="I42" s="31"/>
       <c r="J42" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K42" s="31"/>
       <c r="L42" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="43" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -3125,16 +3101,16 @@
         <v>737</v>
       </c>
       <c r="B43" s="54" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C43" s="44" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D43" s="72" t="s">
         <v>20</v>
       </c>
       <c r="E43" s="45" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="F43" s="46"/>
       <c r="G43" s="46"/>
@@ -3148,10 +3124,10 @@
         <v>952</v>
       </c>
       <c r="B44" s="49" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C44" s="29" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D44" s="20" t="s">
         <v>14</v>
@@ -3160,19 +3136,19 @@
         <v>1847</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G44" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H44" s="31"/>
       <c r="I44" s="31"/>
       <c r="J44" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K44" s="31"/>
       <c r="L44" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="45" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3180,10 +3156,10 @@
         <v>911</v>
       </c>
       <c r="B45" s="28" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C45" s="29" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D45" s="33" t="s">
         <v>17</v>
@@ -3192,15 +3168,15 @@
         <v>184718</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H45" s="31"/>
       <c r="I45" s="31"/>
       <c r="J45" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K45" s="31"/>
     </row>
@@ -3209,10 +3185,10 @@
         <v>878</v>
       </c>
       <c r="B46" s="28" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C46" s="29" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D46" s="33" t="s">
         <v>17</v>
@@ -3221,19 +3197,19 @@
         <v>1847</v>
       </c>
       <c r="F46" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G46" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H46" s="31"/>
       <c r="I46" s="31"/>
       <c r="J46" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K46" s="31"/>
       <c r="L46" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="47" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3241,10 +3217,10 @@
         <v>337</v>
       </c>
       <c r="B47" s="49" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C47" s="33" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D47" s="20" t="s">
         <v>14</v>
@@ -3253,19 +3229,19 @@
         <v>1847</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G47" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H47" s="31"/>
       <c r="I47" s="31"/>
       <c r="J47" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K47" s="31"/>
       <c r="L47" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="48" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -3273,10 +3249,10 @@
         <v>1048</v>
       </c>
       <c r="B48" s="54" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C48" s="44" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D48" s="53" t="s">
         <v>17</v>
@@ -3294,10 +3270,10 @@
         <v>160</v>
       </c>
       <c r="B49" s="28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C49" s="29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D49" s="20" t="s">
         <v>14</v>
@@ -3306,19 +3282,19 @@
         <v>1847</v>
       </c>
       <c r="F49" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G49" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H49" s="31"/>
       <c r="I49" s="31"/>
       <c r="J49" s="31" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="K49" s="31"/>
       <c r="L49" s="32" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="50" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -3326,10 +3302,10 @@
         <v>825</v>
       </c>
       <c r="B50" s="54" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C50" s="44" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D50" s="53" t="s">
         <v>14</v>
@@ -3349,10 +3325,10 @@
         <v>1006</v>
       </c>
       <c r="B51" s="49" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C51" s="33" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D51" s="20" t="s">
         <v>17</v>
@@ -3361,19 +3337,19 @@
         <v>1847</v>
       </c>
       <c r="F51" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G51" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H51" s="31"/>
       <c r="I51" s="31"/>
       <c r="J51" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K51" s="31"/>
       <c r="L51" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3381,10 +3357,10 @@
         <v>943</v>
       </c>
       <c r="B52" s="49" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C52" s="29" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D52" s="20" t="s">
         <v>14</v>
@@ -3393,19 +3369,19 @@
         <v>1847</v>
       </c>
       <c r="F52" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G52" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H52" s="31"/>
       <c r="I52" s="31"/>
       <c r="J52" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K52" s="31"/>
       <c r="L52" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="53" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3413,10 +3389,10 @@
         <v>995</v>
       </c>
       <c r="B53" s="49" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C53" s="29" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D53" s="20" t="s">
         <v>14</v>
@@ -3425,15 +3401,15 @@
         <v>1847</v>
       </c>
       <c r="F53" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G53" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H53" s="31"/>
       <c r="I53" s="31"/>
       <c r="J53" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K53" s="31"/>
     </row>
@@ -3457,10 +3433,10 @@
         <v>249</v>
       </c>
       <c r="B55" s="28" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C55" s="29" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D55" s="33" t="s">
         <v>17</v>
@@ -3469,19 +3445,19 @@
         <v>1847</v>
       </c>
       <c r="F55" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G55" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H55" s="31"/>
       <c r="I55" s="31"/>
       <c r="J55" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K55" s="31"/>
       <c r="L55" s="32" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="56" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3489,10 +3465,10 @@
         <v>287</v>
       </c>
       <c r="B56" s="28" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C56" s="29" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D56" s="33" t="s">
         <v>17</v>
@@ -3501,19 +3477,19 @@
         <v>1847</v>
       </c>
       <c r="F56" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G56" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H56" s="31"/>
       <c r="I56" s="31"/>
       <c r="J56" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K56" s="31"/>
       <c r="L56" s="32" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="57" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3521,10 +3497,10 @@
         <v>790</v>
       </c>
       <c r="B57" s="28" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C57" s="29" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D57" s="20" t="s">
         <v>14</v>
@@ -3533,19 +3509,19 @@
         <v>1847</v>
       </c>
       <c r="F57" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G57" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H57" s="31"/>
       <c r="I57" s="31"/>
       <c r="J57" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K57" s="31"/>
       <c r="L57" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="58" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3553,10 +3529,10 @@
         <v>879</v>
       </c>
       <c r="B58" s="28" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C58" s="29" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D58" s="20" t="s">
         <v>14</v>
@@ -3565,19 +3541,19 @@
         <v>1847</v>
       </c>
       <c r="F58" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G58" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H58" s="31"/>
       <c r="I58" s="31"/>
       <c r="J58" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K58" s="31"/>
       <c r="L58" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="59" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3585,10 +3561,10 @@
         <v>1010</v>
       </c>
       <c r="B59" s="28" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C59" s="29" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D59" s="20" t="s">
         <v>14</v>
@@ -3597,19 +3573,19 @@
         <v>2932</v>
       </c>
       <c r="F59" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G59" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H59" s="31"/>
       <c r="I59" s="31"/>
       <c r="J59" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K59" s="31"/>
       <c r="L59" s="32" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="60" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3617,31 +3593,31 @@
         <v>1024</v>
       </c>
       <c r="B60" s="28" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C60" s="29" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D60" s="20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E60" s="34">
         <v>1847</v>
       </c>
       <c r="F60" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G60" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H60" s="31"/>
       <c r="I60" s="31"/>
       <c r="J60" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K60" s="31"/>
       <c r="L60" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="61" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3649,10 +3625,10 @@
         <v>1007</v>
       </c>
       <c r="B61" s="49" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C61" s="33" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D61" s="20" t="s">
         <v>14</v>
@@ -3661,19 +3637,19 @@
         <v>184718</v>
       </c>
       <c r="F61" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G61" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H61" s="31"/>
       <c r="I61" s="31"/>
       <c r="J61" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K61" s="31"/>
       <c r="L61" s="32" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="62" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3681,10 +3657,10 @@
         <v>116</v>
       </c>
       <c r="B62" s="49" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C62" s="33" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D62" s="20" t="s">
         <v>14</v>
@@ -3693,19 +3669,19 @@
         <v>1847</v>
       </c>
       <c r="F62" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G62" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H62" s="31"/>
       <c r="I62" s="31"/>
       <c r="J62" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K62" s="31"/>
       <c r="L62" s="32" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="63" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3713,10 +3689,10 @@
         <v>969</v>
       </c>
       <c r="B63" s="49" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C63" s="29" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D63" s="20" t="s">
         <v>17</v>
@@ -3725,19 +3701,19 @@
         <v>1847</v>
       </c>
       <c r="F63" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G63" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H63" s="31"/>
       <c r="I63" s="31"/>
       <c r="J63" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K63" s="31"/>
       <c r="L63" s="32" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="64" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3745,10 +3721,10 @@
         <v>817</v>
       </c>
       <c r="B64" s="49" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C64" s="33" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D64" s="20" t="s">
         <v>20</v>
@@ -3757,19 +3733,19 @@
         <v>1847</v>
       </c>
       <c r="F64" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G64" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H64" s="31"/>
       <c r="I64" s="31"/>
       <c r="J64" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K64" s="31"/>
       <c r="L64" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="65" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -3777,10 +3753,10 @@
         <v>903</v>
       </c>
       <c r="B65" s="49" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C65" s="33" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D65" s="20" t="s">
         <v>17</v>
@@ -3789,19 +3765,19 @@
         <v>1847</v>
       </c>
       <c r="F65" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G65" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H65" s="31"/>
       <c r="I65" s="31"/>
       <c r="J65" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K65" s="31"/>
       <c r="L65" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
@@ -3809,10 +3785,10 @@
         <v>987</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D66" s="14" t="s">
         <v>14</v>
@@ -3832,16 +3808,16 @@
         <v>830</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D67" s="14" t="s">
         <v>17</v>
       </c>
       <c r="E67" s="15" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -3855,10 +3831,10 @@
         <v>821</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D68" s="14" t="s">
         <v>20</v>
@@ -3878,10 +3854,10 @@
         <v>446</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D69" s="14" t="s">
         <v>14</v>
@@ -3901,10 +3877,10 @@
         <v>889</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>14</v>
@@ -3924,10 +3900,10 @@
         <v>917</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D71" s="14" t="s">
         <v>17</v>
@@ -3947,10 +3923,10 @@
         <v>528</v>
       </c>
       <c r="B72" s="49" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C72" s="33" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D72" s="20" t="s">
         <v>17</v>
@@ -3959,19 +3935,19 @@
         <v>1847</v>
       </c>
       <c r="F72" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G72" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H72" s="31"/>
       <c r="I72" s="31"/>
       <c r="J72" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K72" s="31"/>
       <c r="L72" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="73" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -3979,16 +3955,16 @@
         <v>245</v>
       </c>
       <c r="B73" s="54" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="C73" s="44" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D73" s="53" t="s">
         <v>14</v>
       </c>
       <c r="E73" s="45" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F73" s="46"/>
       <c r="G73" s="46"/>
@@ -4002,10 +3978,10 @@
         <v>1043</v>
       </c>
       <c r="B74" s="49" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C74" s="33" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D74" s="20" t="s">
         <v>17</v>
@@ -4014,19 +3990,19 @@
         <v>1847</v>
       </c>
       <c r="F74" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G74" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H74" s="31"/>
       <c r="I74" s="31"/>
       <c r="J74" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K74" s="31"/>
       <c r="L74" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="75" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4034,10 +4010,10 @@
         <v>84</v>
       </c>
       <c r="B75" s="28" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C75" s="29" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D75" s="20" t="s">
         <v>14</v>
@@ -4046,19 +4022,19 @@
         <v>1847</v>
       </c>
       <c r="F75" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G75" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="31"/>
       <c r="J75" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K75" s="31"/>
       <c r="L75" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="76" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4066,10 +4042,10 @@
         <v>1003</v>
       </c>
       <c r="B76" s="28" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C76" s="29" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D76" s="20" t="s">
         <v>14</v>
@@ -4078,19 +4054,19 @@
         <v>1847</v>
       </c>
       <c r="F76" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G76" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="31"/>
       <c r="J76" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K76" s="31"/>
       <c r="L76" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="77" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4098,10 +4074,10 @@
         <v>985</v>
       </c>
       <c r="B77" s="49" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C77" s="33" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D77" s="20" t="s">
         <v>14</v>
@@ -4110,19 +4086,19 @@
         <v>1847</v>
       </c>
       <c r="F77" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G77" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H77" s="31"/>
       <c r="I77" s="31"/>
       <c r="J77" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K77" s="31"/>
       <c r="L77" s="32" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="78" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4130,10 +4106,10 @@
         <v>503</v>
       </c>
       <c r="B78" s="79" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C78" s="33" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D78" s="20" t="s">
         <v>14</v>
@@ -4142,19 +4118,19 @@
         <v>1847</v>
       </c>
       <c r="F78" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G78" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="31"/>
       <c r="J78" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K78" s="31"/>
       <c r="L78" s="32" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="79" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4162,10 +4138,10 @@
         <v>1001</v>
       </c>
       <c r="B79" s="74" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C79" s="48" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D79" s="20" t="s">
         <v>17</v>
@@ -4174,19 +4150,19 @@
         <v>184718</v>
       </c>
       <c r="F79" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G79" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="31"/>
       <c r="J79" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K79" s="31"/>
       <c r="L79" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="80" spans="1:12" s="32" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4194,10 +4170,10 @@
         <v>999</v>
       </c>
       <c r="B80" s="75" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C80" s="68" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D80" s="20" t="s">
         <v>17</v>
@@ -4206,19 +4182,19 @@
         <v>1847</v>
       </c>
       <c r="F80" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G80" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="31"/>
       <c r="J80" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K80" s="31"/>
       <c r="L80" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
@@ -4226,10 +4202,10 @@
         <v>902</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D81" s="14" t="s">
         <v>14</v>
@@ -4249,10 +4225,10 @@
         <v>755</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D82" s="14" t="s">
         <v>14</v>
@@ -4266,10 +4242,10 @@
         <v>439</v>
       </c>
       <c r="B83" s="17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D83" s="14" t="s">
         <v>17</v>
@@ -4289,10 +4265,10 @@
         <v>1015</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D84" s="14" t="s">
         <v>14</v>
@@ -4312,10 +4288,10 @@
         <v>508</v>
       </c>
       <c r="B85" s="17" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D85" s="14" t="s">
         <v>14</v>
@@ -4335,10 +4311,10 @@
         <v>123</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D86" s="14" t="s">
         <v>14</v>
@@ -4358,10 +4334,10 @@
         <v>946</v>
       </c>
       <c r="B87" s="49" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C87" s="68" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D87" s="20" t="s">
         <v>14</v>
@@ -4370,19 +4346,19 @@
         <v>184718</v>
       </c>
       <c r="F87" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G87" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H87" s="31"/>
       <c r="I87" s="31"/>
       <c r="J87" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K87" s="31"/>
       <c r="L87" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
@@ -4390,10 +4366,10 @@
         <v>35</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D88" s="14" t="s">
         <v>14</v>
@@ -4413,10 +4389,10 @@
         <v>101</v>
       </c>
       <c r="B89" s="28" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C89" s="29" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D89" s="20" t="s">
         <v>14</v>
@@ -4425,19 +4401,19 @@
         <v>1847</v>
       </c>
       <c r="F89" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G89" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H89" s="31"/>
       <c r="I89" s="31"/>
       <c r="J89" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K89" s="31"/>
       <c r="L89" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
@@ -4445,16 +4421,16 @@
         <v>1037</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C90" s="12" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D90" s="14" t="s">
         <v>14</v>
       </c>
       <c r="E90" s="15" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
@@ -4468,10 +4444,10 @@
         <v>707</v>
       </c>
       <c r="B91" s="17" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D91" s="14" t="s">
         <v>14</v>
@@ -4491,10 +4467,10 @@
         <v>804</v>
       </c>
       <c r="B92" s="49" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C92" s="33" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D92" s="20" t="s">
         <v>20</v>
@@ -4503,15 +4479,15 @@
         <v>1847</v>
       </c>
       <c r="F92" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G92" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H92" s="31"/>
       <c r="I92" s="31"/>
       <c r="J92" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K92" s="31"/>
     </row>
@@ -4520,10 +4496,10 @@
         <v>1020</v>
       </c>
       <c r="B93" s="22" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C93" s="13" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>14</v>
@@ -4543,10 +4519,10 @@
         <v>1022</v>
       </c>
       <c r="B94" s="22" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C94" s="13" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D94" s="14" t="s">
         <v>14</v>
@@ -4579,13 +4555,13 @@
         <v>1023</v>
       </c>
       <c r="B96" s="23" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C96" s="13" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D96" s="14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E96" s="15">
         <v>1847</v>
@@ -4602,10 +4578,10 @@
         <v>97</v>
       </c>
       <c r="B97" s="28" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C97" s="29" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D97" s="20" t="s">
         <v>14</v>
@@ -4614,19 +4590,19 @@
         <v>1847</v>
       </c>
       <c r="F97" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G97" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H97" s="31"/>
       <c r="I97" s="31"/>
       <c r="J97" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K97" s="31"/>
       <c r="L97" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
@@ -4634,10 +4610,10 @@
         <v>1044</v>
       </c>
       <c r="B98" s="24" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>20</v>
@@ -4657,10 +4633,10 @@
         <v>67</v>
       </c>
       <c r="B99" s="17" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C99" s="13" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D99" s="14" t="s">
         <v>17</v>
@@ -4695,10 +4671,10 @@
         <v>916</v>
       </c>
       <c r="B101" s="79" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="C101" s="66" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D101" s="48" t="s">
         <v>17</v>
@@ -4707,19 +4683,19 @@
         <v>612435</v>
       </c>
       <c r="F101" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G101" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H101" s="31"/>
       <c r="I101" s="31"/>
       <c r="J101" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K101" s="31"/>
       <c r="L101" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
@@ -4727,10 +4703,10 @@
         <v>1019</v>
       </c>
       <c r="B102" s="21" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C102" s="25" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D102" s="16" t="s">
         <v>14</v>
@@ -4750,10 +4726,10 @@
         <v>948</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="C103" s="19" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D103" s="14" t="s">
         <v>20</v>
@@ -4773,10 +4749,10 @@
         <v>989</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C104" s="19" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D104" s="14" t="s">
         <v>17</v>
@@ -4811,10 +4787,10 @@
         <v>814</v>
       </c>
       <c r="B106" s="49" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C106" s="29" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D106" s="20" t="s">
         <v>14</v>
@@ -4823,19 +4799,19 @@
         <v>1847</v>
       </c>
       <c r="F106" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G106" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H106" s="31"/>
       <c r="I106" s="31"/>
       <c r="J106" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K106" s="31"/>
       <c r="L106" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="107" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4843,10 +4819,10 @@
         <v>856</v>
       </c>
       <c r="B107" s="49" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C107" s="33" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>17</v>
@@ -4855,19 +4831,19 @@
         <v>3879</v>
       </c>
       <c r="F107" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G107" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H107" s="31"/>
       <c r="I107" s="31"/>
       <c r="J107" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K107" s="31"/>
       <c r="L107" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="108" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -4931,10 +4907,10 @@
         <v>403</v>
       </c>
       <c r="B112" s="28" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C112" s="33" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D112" s="20" t="s">
         <v>14</v>
@@ -4943,19 +4919,19 @@
         <v>1847</v>
       </c>
       <c r="F112" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G112" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H112" s="31"/>
       <c r="I112" s="31"/>
       <c r="J112" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K112" s="31"/>
       <c r="L112" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="113" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -4963,10 +4939,10 @@
         <v>935</v>
       </c>
       <c r="B113" s="28" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C113" s="68" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D113" s="20" t="s">
         <v>14</v>
@@ -4975,19 +4951,19 @@
         <v>184718</v>
       </c>
       <c r="F113" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G113" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H113" s="31"/>
       <c r="I113" s="31"/>
       <c r="J113" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K113" s="31"/>
       <c r="L113" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="114" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -5008,10 +4984,10 @@
         <v>3</v>
       </c>
       <c r="B115" s="77" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C115" s="78" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D115" s="61" t="s">
         <v>14</v>
@@ -5020,22 +4996,22 @@
         <v>1847</v>
       </c>
       <c r="F115" s="63" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G115" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H115" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="I115" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="J115" s="63" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K115" s="63" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="116" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5043,10 +5019,10 @@
         <v>837</v>
       </c>
       <c r="B116" s="28" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C116" s="29" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D116" s="20" t="s">
         <v>14</v>
@@ -5055,19 +5031,19 @@
         <v>1847</v>
       </c>
       <c r="F116" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G116" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H116" s="31"/>
       <c r="I116" s="31"/>
       <c r="J116" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K116" s="31"/>
       <c r="L116" s="32" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="117" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5075,10 +5051,10 @@
         <v>973</v>
       </c>
       <c r="B117" s="28" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C117" s="29" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D117" s="20" t="s">
         <v>17</v>
@@ -5087,19 +5063,19 @@
         <v>184718</v>
       </c>
       <c r="F117" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G117" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H117" s="31"/>
       <c r="I117" s="31"/>
       <c r="J117" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K117" s="31"/>
       <c r="L117" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="118" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -5120,10 +5096,10 @@
         <v>34</v>
       </c>
       <c r="B119" s="28" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C119" s="29" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D119" s="20" t="s">
         <v>14</v>
@@ -5132,19 +5108,19 @@
         <v>1246</v>
       </c>
       <c r="F119" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G119" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H119" s="31"/>
       <c r="I119" s="31"/>
       <c r="J119" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K119" s="31"/>
       <c r="L119" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
@@ -5152,10 +5128,10 @@
         <v>1016</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D120" s="14" t="s">
         <v>17</v>
@@ -5175,10 +5151,10 @@
         <v>92</v>
       </c>
       <c r="B121" s="11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C121" s="12" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D121" s="14" t="s">
         <v>14</v>
@@ -5198,10 +5174,10 @@
         <v>753</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C122" s="12" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D122" s="14" t="s">
         <v>20</v>
@@ -5221,10 +5197,10 @@
         <v>970</v>
       </c>
       <c r="B123" s="11" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C123" s="12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D123" s="14" t="s">
         <v>14</v>
@@ -5244,10 +5220,10 @@
         <v>525</v>
       </c>
       <c r="B124" s="17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C124" s="13" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D124" s="14" t="s">
         <v>17</v>
@@ -5306,10 +5282,10 @@
         <v>183</v>
       </c>
       <c r="B128" s="28" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D128" s="20" t="s">
         <v>17</v>
@@ -5318,15 +5294,15 @@
         <v>1847</v>
       </c>
       <c r="F128" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G128" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H128" s="31"/>
       <c r="I128" s="31"/>
       <c r="J128" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K128" s="31"/>
     </row>
@@ -5335,10 +5311,10 @@
         <v>793</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C129" s="12" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D129" s="14" t="s">
         <v>14</v>
@@ -5358,10 +5334,10 @@
         <v>24</v>
       </c>
       <c r="B130" s="17" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C130" s="12" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D130" s="14" t="s">
         <v>20</v>
@@ -5381,10 +5357,10 @@
         <v>71</v>
       </c>
       <c r="B131" s="17" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C131" s="13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D131" s="14" t="s">
         <v>20</v>
@@ -5430,16 +5406,16 @@
         <v>1000</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C134" s="19" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D134" s="14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E134" s="15" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F134" s="3"/>
       <c r="G134" s="3"/>
@@ -5453,10 +5429,10 @@
         <v>57</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C135" s="13" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D135" s="14" t="s">
         <v>17</v>
@@ -5476,10 +5452,10 @@
         <v>941</v>
       </c>
       <c r="B136" s="17" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C136" s="12" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D136" s="14" t="s">
         <v>14</v>
@@ -5499,10 +5475,10 @@
         <v>505</v>
       </c>
       <c r="B137" s="49" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C137" s="33" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D137" s="20" t="s">
         <v>14</v>
@@ -5511,19 +5487,19 @@
         <v>1847</v>
       </c>
       <c r="F137" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G137" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H137" s="31"/>
       <c r="I137" s="31"/>
       <c r="J137" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K137" s="31"/>
       <c r="L137" s="32" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="138" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5531,31 +5507,31 @@
         <v>931</v>
       </c>
       <c r="B138" s="49" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="C138" s="68" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D138" s="20" t="s">
         <v>14</v>
       </c>
       <c r="E138" s="34" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F138" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G138" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H138" s="31"/>
       <c r="I138" s="31"/>
       <c r="J138" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K138" s="31"/>
       <c r="L138" s="32" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
     </row>
     <row r="139" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5569,7 +5545,7 @@
       <c r="H139" s="31"/>
       <c r="I139" s="31"/>
       <c r="J139" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K139" s="31"/>
     </row>
@@ -5578,10 +5554,10 @@
         <v>802</v>
       </c>
       <c r="B140" s="28" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C140" s="29" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D140" s="33" t="s">
         <v>17</v>
@@ -5590,19 +5566,19 @@
         <v>1847</v>
       </c>
       <c r="F140" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G140" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H140" s="31"/>
       <c r="I140" s="31"/>
       <c r="J140" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K140" s="31"/>
       <c r="L140" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="141" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5610,31 +5586,31 @@
         <v>1035</v>
       </c>
       <c r="B141" s="28" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C141" s="29" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D141" s="33" t="s">
         <v>14</v>
       </c>
       <c r="E141" s="34" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F141" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G141" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H141" s="31"/>
       <c r="I141" s="31"/>
       <c r="J141" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K141" s="31"/>
       <c r="L141" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="142" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5642,10 +5618,10 @@
         <v>944</v>
       </c>
       <c r="B142" s="49" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C142" s="29" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D142" s="20" t="s">
         <v>14</v>
@@ -5654,19 +5630,19 @@
         <v>1847</v>
       </c>
       <c r="F142" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G142" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H142" s="31"/>
       <c r="I142" s="31"/>
       <c r="J142" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K142" s="31"/>
       <c r="L142" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="143" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -5713,10 +5689,10 @@
         <v>910</v>
       </c>
       <c r="B146" s="49" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C146" s="33" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D146" s="20" t="s">
         <v>20</v>
@@ -5725,19 +5701,19 @@
         <v>1847</v>
       </c>
       <c r="F146" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G146" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H146" s="31"/>
       <c r="I146" s="31"/>
       <c r="J146" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K146" s="31"/>
       <c r="L146" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="147" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5745,10 +5721,10 @@
         <v>820</v>
       </c>
       <c r="B147" s="28" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C147" s="29" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D147" s="20" t="s">
         <v>14</v>
@@ -5757,19 +5733,19 @@
         <v>1847</v>
       </c>
       <c r="F147" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G147" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H147" s="31"/>
       <c r="I147" s="31"/>
       <c r="J147" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K147" s="31"/>
       <c r="L147" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="148" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5777,10 +5753,10 @@
         <v>152</v>
       </c>
       <c r="B148" s="28" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C148" s="29" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D148" s="20" t="s">
         <v>14</v>
@@ -5789,19 +5765,19 @@
         <v>1847</v>
       </c>
       <c r="F148" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G148" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H148" s="31"/>
       <c r="I148" s="31"/>
       <c r="J148" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K148" s="31"/>
       <c r="L148" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="149" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5809,10 +5785,10 @@
         <v>148</v>
       </c>
       <c r="B149" s="28" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C149" s="29" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D149" s="33" t="s">
         <v>17</v>
@@ -5821,19 +5797,19 @@
         <v>1847</v>
       </c>
       <c r="F149" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G149" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H149" s="31"/>
       <c r="I149" s="31"/>
       <c r="J149" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K149" s="31"/>
       <c r="L149" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="150" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5841,10 +5817,10 @@
         <v>992</v>
       </c>
       <c r="B150" s="28" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C150" s="29" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D150" s="33" t="s">
         <v>14</v>
@@ -5853,19 +5829,19 @@
         <v>184718</v>
       </c>
       <c r="F150" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G150" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H150" s="31"/>
       <c r="I150" s="31"/>
       <c r="J150" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K150" s="31"/>
       <c r="L150" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="151" spans="1:13" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -5886,10 +5862,10 @@
         <v>419</v>
       </c>
       <c r="B152" s="28" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C152" s="29" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D152" s="20" t="s">
         <v>14</v>
@@ -5898,19 +5874,19 @@
         <v>1348</v>
       </c>
       <c r="F152" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G152" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H152" s="31"/>
       <c r="I152" s="31"/>
       <c r="J152" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K152" s="31"/>
       <c r="L152" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="153" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5918,10 +5894,10 @@
         <v>99</v>
       </c>
       <c r="B153" s="28" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C153" s="29" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D153" s="20" t="s">
         <v>14</v>
@@ -5930,22 +5906,22 @@
         <v>1847</v>
       </c>
       <c r="F153" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G153" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H153" s="31"/>
       <c r="I153" s="31"/>
       <c r="J153" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K153" s="31"/>
       <c r="L153" s="32" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="M153" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="154" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5953,10 +5929,10 @@
         <v>811</v>
       </c>
       <c r="B154" s="28" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C154" s="29" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D154" s="20" t="s">
         <v>14</v>
@@ -5965,19 +5941,19 @@
         <v>184718</v>
       </c>
       <c r="F154" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G154" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H154" s="31"/>
       <c r="I154" s="31"/>
       <c r="J154" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K154" s="31"/>
       <c r="L154" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="155" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -5985,10 +5961,10 @@
         <v>131</v>
       </c>
       <c r="B155" s="28" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C155" s="29" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D155" s="33" t="s">
         <v>17</v>
@@ -5997,19 +5973,19 @@
         <v>184718</v>
       </c>
       <c r="F155" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G155" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H155" s="31"/>
       <c r="I155" s="31"/>
       <c r="J155" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K155" s="31"/>
       <c r="L155" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="156" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6017,10 +5993,10 @@
         <v>835</v>
       </c>
       <c r="B156" s="28" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C156" s="29" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D156" s="20" t="s">
         <v>14</v>
@@ -6029,19 +6005,19 @@
         <v>1847</v>
       </c>
       <c r="F156" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G156" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H156" s="31"/>
       <c r="I156" s="31"/>
       <c r="J156" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K156" s="31"/>
       <c r="L156" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="157" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6049,10 +6025,10 @@
         <v>448</v>
       </c>
       <c r="B157" s="28" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C157" s="29" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D157" s="33" t="s">
         <v>17</v>
@@ -6061,19 +6037,19 @@
         <v>1847</v>
       </c>
       <c r="F157" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G157" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H157" s="31"/>
       <c r="I157" s="31"/>
       <c r="J157" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K157" s="31"/>
       <c r="L157" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="158" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6081,10 +6057,10 @@
         <v>1018</v>
       </c>
       <c r="B158" s="28" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C158" s="29" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D158" s="33" t="s">
         <v>20</v>
@@ -6093,19 +6069,19 @@
         <v>1847</v>
       </c>
       <c r="F158" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G158" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H158" s="31"/>
       <c r="I158" s="31"/>
       <c r="J158" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K158" s="31"/>
       <c r="L158" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="159" spans="1:13" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6113,10 +6089,10 @@
         <v>367</v>
       </c>
       <c r="B159" s="28" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C159" s="29" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D159" s="20" t="s">
         <v>14</v>
@@ -6125,15 +6101,15 @@
         <v>184718</v>
       </c>
       <c r="F159" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G159" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H159" s="31"/>
       <c r="I159" s="31"/>
       <c r="J159" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K159" s="31"/>
     </row>
@@ -6168,10 +6144,10 @@
         <v>789</v>
       </c>
       <c r="B162" s="49" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C162" s="33" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D162" s="20" t="s">
         <v>14</v>
@@ -6180,19 +6156,19 @@
         <v>1847</v>
       </c>
       <c r="F162" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G162" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H162" s="31"/>
       <c r="I162" s="31"/>
       <c r="J162" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K162" s="31"/>
       <c r="L162" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="163" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6200,10 +6176,10 @@
         <v>1039</v>
       </c>
       <c r="B163" s="49" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C163" s="33" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D163" s="20" t="s">
         <v>17</v>
@@ -6212,19 +6188,19 @@
         <v>184718</v>
       </c>
       <c r="F163" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G163" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H163" s="31"/>
       <c r="I163" s="31"/>
       <c r="J163" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K163" s="31"/>
       <c r="L163" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="164" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6232,10 +6208,10 @@
         <v>742</v>
       </c>
       <c r="B164" s="28" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C164" s="29" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D164" s="20" t="s">
         <v>14</v>
@@ -6244,19 +6220,19 @@
         <v>1847</v>
       </c>
       <c r="F164" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G164" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H164" s="31"/>
       <c r="I164" s="31"/>
       <c r="J164" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K164" s="31"/>
       <c r="L164" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="165" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6264,10 +6240,10 @@
         <v>9</v>
       </c>
       <c r="B165" s="49" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C165" s="33" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D165" s="20" t="s">
         <v>17</v>
@@ -6276,19 +6252,19 @@
         <v>1847</v>
       </c>
       <c r="F165" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G165" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H165" s="31"/>
       <c r="I165" s="31"/>
       <c r="J165" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K165" s="31"/>
       <c r="L165" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="166" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6296,10 +6272,10 @@
         <v>993</v>
       </c>
       <c r="B166" s="28" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C166" s="29" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D166" s="33" t="s">
         <v>17</v>
@@ -6308,19 +6284,19 @@
         <v>1847</v>
       </c>
       <c r="F166" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G166" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H166" s="31"/>
       <c r="I166" s="31"/>
       <c r="J166" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K166" s="31"/>
       <c r="L166" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="167" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6328,31 +6304,31 @@
         <v>342</v>
       </c>
       <c r="B167" s="28" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D167" s="33" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E167" s="34">
         <v>1847</v>
       </c>
       <c r="F167" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G167" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H167" s="31"/>
       <c r="I167" s="31"/>
       <c r="J167" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K167" s="31"/>
       <c r="L167" s="32" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
     </row>
     <row r="168" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -6373,10 +6349,10 @@
         <v>744</v>
       </c>
       <c r="B169" s="28" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C169" s="29" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D169" s="33" t="s">
         <v>17</v>
@@ -6385,19 +6361,19 @@
         <v>1847</v>
       </c>
       <c r="F169" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G169" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H169" s="31"/>
       <c r="I169" s="31"/>
       <c r="J169" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K169" s="31"/>
       <c r="L169" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="170" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6405,10 +6381,10 @@
         <v>907</v>
       </c>
       <c r="B170" s="28" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D170" s="20" t="s">
         <v>14</v>
@@ -6417,19 +6393,19 @@
         <v>2232</v>
       </c>
       <c r="F170" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G170" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H170" s="31"/>
       <c r="I170" s="31"/>
       <c r="J170" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K170" s="31"/>
       <c r="L170" s="32" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="171" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -6476,10 +6452,10 @@
         <v>283</v>
       </c>
       <c r="B174" s="28" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C174" s="29" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D174" s="20" t="s">
         <v>20</v>
@@ -6488,19 +6464,19 @@
         <v>1847</v>
       </c>
       <c r="F174" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G174" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H174" s="31"/>
       <c r="I174" s="31"/>
       <c r="J174" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K174" s="31"/>
       <c r="L174" s="32" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="175" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6508,10 +6484,10 @@
         <v>170</v>
       </c>
       <c r="B175" s="28" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D175" s="20" t="s">
         <v>14</v>
@@ -6520,19 +6496,19 @@
         <v>1847</v>
       </c>
       <c r="F175" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G175" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H175" s="31"/>
       <c r="I175" s="31"/>
       <c r="J175" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K175" s="31"/>
       <c r="L175" s="32" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="176" spans="1:12" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -6540,10 +6516,10 @@
         <v>502</v>
       </c>
       <c r="B176" s="28" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D176" s="33" t="s">
         <v>17</v>
@@ -6552,19 +6528,19 @@
         <v>1847</v>
       </c>
       <c r="F176" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G176" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="H176" s="31"/>
       <c r="I176" s="31"/>
       <c r="J176" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="K176" s="31"/>
       <c r="L176" s="32" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="177" spans="1:12" s="47" customFormat="1" x14ac:dyDescent="0.25">
@@ -6598,10 +6574,10 @@
         <v>136</v>
       </c>
       <c r="B179" s="28" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C179" s="29" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D179" s="48" t="s">
         <v>17</v>
@@ -6610,15 +6586,15 @@
         <v>1847</v>
       </c>
       <c r="F179" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G179" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H179" s="31"/>
       <c r="I179" s="31"/>
       <c r="J179" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K179" s="31"/>
     </row>
@@ -6627,10 +6603,10 @@
         <v>895</v>
       </c>
       <c r="B180" s="28" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C180" s="29" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D180" s="33" t="s">
         <v>14</v>
@@ -6639,19 +6615,19 @@
         <v>184718</v>
       </c>
       <c r="F180" s="31" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="G180" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="H180" s="31"/>
       <c r="I180" s="31"/>
       <c r="J180" s="31" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="K180" s="31"/>
       <c r="L180" s="32" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>